<commit_message>
Add PDF reporting and deployment updates
</commit_message>
<xml_diff>
--- a/SampleData/All Metrics Cleaned.xlsx
+++ b/SampleData/All Metrics Cleaned.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rod_w\OneDrive\PythonStuff\Reliability\SampleData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4534e0d33770ad0c/PythonStuff/Reliability/SampleData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51348253-1831-42C8-A93C-7BB9342745BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{51348253-1831-42C8-A93C-7BB9342745BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51DD789A-4DB2-4A0E-8AC4-EC2E637AAA11}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{18937AAF-621B-4514-A62F-915B9E134D21}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="121">
   <si>
     <t>BRENDAN_1</t>
   </si>
@@ -983,10 +983,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545F92D5-595F-47A7-BE29-23CA89498328}">
-  <dimension ref="A1:BU7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:73" s="1" customFormat="1" ht="72.5">
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="58">
       <c r="A1" s="1">
         <v>0</v>
       </c>
@@ -1008,206 +1008,8 @@
       <c r="G1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="Z1" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AF1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="AG1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="AH1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="AI1" s="1">
-        <v>0</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AP1" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="AQ1" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="AR1" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="AS1" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="AT1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AU1" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="AV1" s="5">
-        <v>0</v>
-      </c>
-      <c r="AW1" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="AX1" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="AY1" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="AZ1" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="BA1" s="1">
-        <v>0</v>
-      </c>
-      <c r="BB1" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="BC1" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="BE1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="BF1" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="BG1" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="BH1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="BI1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="BJ1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BK1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BL1" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="BM1" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="BN1" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="BO1" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="BP1" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="BQ1" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="BR1" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="BS1" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="BT1" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="BU1" s="2" t="s">
-        <v>82</v>
-      </c>
     </row>
-    <row r="2" spans="1:73">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1229,206 +1031,8 @@
       <c r="G2">
         <v>-23.378299999999999</v>
       </c>
-      <c r="H2">
-        <v>11.928100000000001</v>
-      </c>
-      <c r="I2">
-        <v>10.561299999999999</v>
-      </c>
-      <c r="J2">
-        <v>-25.131599999999999</v>
-      </c>
-      <c r="K2">
-        <v>-29.4681</v>
-      </c>
-      <c r="L2">
-        <v>2.0804</v>
-      </c>
-      <c r="M2">
-        <v>3.7534999999999998</v>
-      </c>
-      <c r="N2">
-        <v>-4.9992000000000001</v>
-      </c>
-      <c r="O2">
-        <v>-8.3742000000000001</v>
-      </c>
-      <c r="P2">
-        <v>16.284700000000001</v>
-      </c>
-      <c r="Q2">
-        <v>15.870200000000001</v>
-      </c>
-      <c r="R2">
-        <v>-26.481200000000001</v>
-      </c>
-      <c r="S2">
-        <v>-20.981300000000001</v>
-      </c>
-      <c r="T2">
-        <v>13.1684</v>
-      </c>
-      <c r="U2">
-        <v>10.613799999999999</v>
-      </c>
-      <c r="V2">
-        <v>-33.542999999999999</v>
-      </c>
-      <c r="W2">
-        <v>-30.444700000000001</v>
-      </c>
-      <c r="X2">
-        <v>3.9123999999999999</v>
-      </c>
-      <c r="Y2">
-        <v>4.5091000000000001</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA2">
-        <v>-1.6199999999999999E-2</v>
-      </c>
-      <c r="AB2">
-        <v>-2.4199999999999999E-2</v>
-      </c>
-      <c r="AC2">
-        <v>0.39190000000000003</v>
-      </c>
-      <c r="AD2">
-        <v>0.39600000000000002</v>
-      </c>
-      <c r="AE2">
-        <v>-3.6999999999999998E-2</v>
-      </c>
-      <c r="AF2">
-        <v>-3.5499999999999997E-2</v>
-      </c>
-      <c r="AG2">
-        <v>0.39779999999999999</v>
-      </c>
-      <c r="AH2">
-        <v>0.40150000000000002</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>52</v>
-      </c>
-      <c r="AJ2">
-        <v>-3.8144999999999998</v>
-      </c>
-      <c r="AK2">
-        <v>-3.5882000000000001</v>
-      </c>
-      <c r="AL2">
-        <v>-2.0373000000000001</v>
-      </c>
-      <c r="AM2">
-        <v>-2.0428999999999999</v>
-      </c>
-      <c r="AN2">
-        <v>-2.6627999999999998</v>
-      </c>
-      <c r="AO2">
-        <v>-2.7136</v>
-      </c>
-      <c r="AP2">
-        <v>-3.8502999999999998</v>
-      </c>
-      <c r="AQ2">
-        <v>-3.7909999999999999</v>
-      </c>
-      <c r="AR2">
-        <v>-1.958</v>
-      </c>
-      <c r="AS2">
-        <v>-1.7813000000000001</v>
-      </c>
-      <c r="AT2">
-        <v>-2.8466999999999998</v>
-      </c>
-      <c r="AU2">
-        <v>-2.6913999999999998</v>
-      </c>
-      <c r="AV2" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="AW2" s="7">
-        <v>675.31470000000002</v>
-      </c>
-      <c r="AX2" s="7">
-        <v>674.57069999999999</v>
-      </c>
-      <c r="AY2" s="7">
-        <v>599.7319</v>
-      </c>
-      <c r="AZ2" s="7">
-        <v>618.54300000000001</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>0</v>
-      </c>
-      <c r="BB2" s="13">
-        <v>9.6296999999999997</v>
-      </c>
-      <c r="BC2" s="13">
-        <v>10.4316</v>
-      </c>
-      <c r="BD2">
-        <v>26.879200000000001</v>
-      </c>
-      <c r="BE2">
-        <v>25.423500000000001</v>
-      </c>
-      <c r="BF2" s="13">
-        <v>9.6463999999999999</v>
-      </c>
-      <c r="BG2" s="13">
-        <v>10.098000000000001</v>
-      </c>
-      <c r="BH2">
-        <v>114.97799999999999</v>
-      </c>
-      <c r="BI2">
-        <v>112.5474</v>
-      </c>
-      <c r="BJ2" s="8">
-        <v>40.025700000000001</v>
-      </c>
-      <c r="BK2" s="8">
-        <v>39.323999999999998</v>
-      </c>
-      <c r="BL2" s="13">
-        <v>13.0137</v>
-      </c>
-      <c r="BM2" s="13">
-        <v>13.0822</v>
-      </c>
-      <c r="BN2">
-        <v>26.946300000000001</v>
-      </c>
-      <c r="BO2">
-        <v>25.3993</v>
-      </c>
-      <c r="BP2" s="13">
-        <v>10.4245</v>
-      </c>
-      <c r="BQ2" s="13">
-        <v>11.3695</v>
-      </c>
-      <c r="BR2">
-        <v>106.0836</v>
-      </c>
-      <c r="BS2">
-        <v>106.1178</v>
-      </c>
-      <c r="BT2" s="8">
-        <v>41.130600000000001</v>
-      </c>
-      <c r="BU2" s="8">
-        <v>39.864400000000003</v>
-      </c>
     </row>
-    <row r="3" spans="1:73">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1450,206 +1054,8 @@
       <c r="G3">
         <v>-30.5733</v>
       </c>
-      <c r="H3">
-        <v>9.8308999999999997</v>
-      </c>
-      <c r="I3">
-        <v>9.4831000000000003</v>
-      </c>
-      <c r="J3">
-        <v>-40.819600000000001</v>
-      </c>
-      <c r="K3">
-        <v>-36.913499999999999</v>
-      </c>
-      <c r="L3">
-        <v>11.6105</v>
-      </c>
-      <c r="M3">
-        <v>11.631600000000001</v>
-      </c>
-      <c r="N3">
-        <v>-6.9448999999999996</v>
-      </c>
-      <c r="O3">
-        <v>-10.5078</v>
-      </c>
-      <c r="P3">
-        <v>24.020700000000001</v>
-      </c>
-      <c r="Q3">
-        <v>24.444299999999998</v>
-      </c>
-      <c r="R3">
-        <v>-35.100299999999997</v>
-      </c>
-      <c r="S3">
-        <v>-34.525199999999998</v>
-      </c>
-      <c r="T3">
-        <v>9.2903000000000002</v>
-      </c>
-      <c r="U3">
-        <v>8.2186000000000003</v>
-      </c>
-      <c r="V3">
-        <v>-36.6907</v>
-      </c>
-      <c r="W3">
-        <v>-29.194400000000002</v>
-      </c>
-      <c r="X3">
-        <v>12.4528</v>
-      </c>
-      <c r="Y3">
-        <v>12.9825</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>1</v>
-      </c>
-      <c r="AA3">
-        <v>-0.1288</v>
-      </c>
-      <c r="AB3">
-        <v>-0.1363</v>
-      </c>
-      <c r="AC3">
-        <v>0.42720000000000002</v>
-      </c>
-      <c r="AD3">
-        <v>0.42620000000000002</v>
-      </c>
-      <c r="AE3">
-        <v>-0.126</v>
-      </c>
-      <c r="AF3">
-        <v>-0.12659999999999999</v>
-      </c>
-      <c r="AG3">
-        <v>0.42109999999999997</v>
-      </c>
-      <c r="AH3">
-        <v>0.42659999999999998</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AJ3">
-        <v>-4.6233000000000004</v>
-      </c>
-      <c r="AK3">
-        <v>-4.5065999999999997</v>
-      </c>
-      <c r="AL3">
-        <v>-2.1429999999999998</v>
-      </c>
-      <c r="AM3">
-        <v>-2.0706000000000002</v>
-      </c>
-      <c r="AN3">
-        <v>-3.0356000000000001</v>
-      </c>
-      <c r="AO3">
-        <v>-3.0070000000000001</v>
-      </c>
-      <c r="AP3">
-        <v>-4.5590000000000002</v>
-      </c>
-      <c r="AQ3">
-        <v>-4.6566999999999998</v>
-      </c>
-      <c r="AR3">
-        <v>-2.0731000000000002</v>
-      </c>
-      <c r="AS3">
-        <v>-2.1612</v>
-      </c>
-      <c r="AT3">
-        <v>-2.3237000000000001</v>
-      </c>
-      <c r="AU3">
-        <v>-2.7128999999999999</v>
-      </c>
-      <c r="AV3" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="AW3" s="7">
-        <v>693.98630000000003</v>
-      </c>
-      <c r="AX3" s="7">
-        <v>690.19129999999996</v>
-      </c>
-      <c r="AY3" s="7">
-        <v>711.6309</v>
-      </c>
-      <c r="AZ3" s="7">
-        <v>694.59199999999998</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>1</v>
-      </c>
-      <c r="BB3" s="13">
-        <v>-1.8280000000000001</v>
-      </c>
-      <c r="BC3" s="13">
-        <v>-2.3900999999999999</v>
-      </c>
-      <c r="BD3">
-        <v>24.877600000000001</v>
-      </c>
-      <c r="BE3">
-        <v>23.7136</v>
-      </c>
-      <c r="BF3" s="13">
-        <v>15.472</v>
-      </c>
-      <c r="BG3" s="13">
-        <v>13.755800000000001</v>
-      </c>
-      <c r="BH3">
-        <v>117.4551</v>
-      </c>
-      <c r="BI3">
-        <v>117.16930000000001</v>
-      </c>
-      <c r="BJ3" s="8">
-        <v>42.975000000000001</v>
-      </c>
-      <c r="BK3" s="8">
-        <v>41.198300000000003</v>
-      </c>
-      <c r="BL3" s="13">
-        <v>-0.89870000000000005</v>
-      </c>
-      <c r="BM3" s="13">
-        <v>-1.2849999999999999</v>
-      </c>
-      <c r="BN3">
-        <v>22.968800000000002</v>
-      </c>
-      <c r="BO3">
-        <v>25.115400000000001</v>
-      </c>
-      <c r="BP3" s="13">
-        <v>15.6799</v>
-      </c>
-      <c r="BQ3" s="13">
-        <v>14.928100000000001</v>
-      </c>
-      <c r="BR3">
-        <v>120.6657</v>
-      </c>
-      <c r="BS3">
-        <v>119.6931</v>
-      </c>
-      <c r="BT3" s="8">
-        <v>38.832999999999998</v>
-      </c>
-      <c r="BU3" s="8">
-        <v>40.686999999999998</v>
-      </c>
     </row>
-    <row r="4" spans="1:73">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1671,206 +1077,8 @@
       <c r="G4">
         <v>-34.686599999999999</v>
       </c>
-      <c r="H4">
-        <v>7.2828999999999997</v>
-      </c>
-      <c r="I4">
-        <v>9.4208999999999996</v>
-      </c>
-      <c r="J4">
-        <v>-38.206400000000002</v>
-      </c>
-      <c r="K4">
-        <v>-30.507200000000001</v>
-      </c>
-      <c r="L4">
-        <v>11.2136</v>
-      </c>
-      <c r="M4">
-        <v>12.63</v>
-      </c>
-      <c r="N4">
-        <v>-4.2774999999999999</v>
-      </c>
-      <c r="O4">
-        <v>-8.5509000000000004</v>
-      </c>
-      <c r="P4">
-        <v>19.466699999999999</v>
-      </c>
-      <c r="Q4">
-        <v>21.459800000000001</v>
-      </c>
-      <c r="R4">
-        <v>-33.9343</v>
-      </c>
-      <c r="S4">
-        <v>-32.490499999999997</v>
-      </c>
-      <c r="T4">
-        <v>12.760999999999999</v>
-      </c>
-      <c r="U4">
-        <v>10.961600000000001</v>
-      </c>
-      <c r="V4">
-        <v>-48.528599999999997</v>
-      </c>
-      <c r="W4">
-        <v>-33.357799999999997</v>
-      </c>
-      <c r="X4">
-        <v>11.693199999999999</v>
-      </c>
-      <c r="Y4">
-        <v>10.857200000000001</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>2</v>
-      </c>
-      <c r="AA4">
-        <v>-0.1401</v>
-      </c>
-      <c r="AB4">
-        <v>-0.1308</v>
-      </c>
-      <c r="AC4">
-        <v>0.4088</v>
-      </c>
-      <c r="AD4">
-        <v>0.40400000000000003</v>
-      </c>
-      <c r="AE4">
-        <v>-0.12089999999999999</v>
-      </c>
-      <c r="AF4">
-        <v>-0.1249</v>
-      </c>
-      <c r="AG4">
-        <v>0.41909999999999997</v>
-      </c>
-      <c r="AH4">
-        <v>0.41610000000000003</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>54</v>
-      </c>
-      <c r="AJ4">
-        <v>-4.2512999999999996</v>
-      </c>
-      <c r="AK4">
-        <v>-4.4954000000000001</v>
-      </c>
-      <c r="AL4">
-        <v>-1.6117999999999999</v>
-      </c>
-      <c r="AM4">
-        <v>-1.8099000000000001</v>
-      </c>
-      <c r="AN4">
-        <v>-2.3860999999999999</v>
-      </c>
-      <c r="AO4">
-        <v>-2.4702999999999999</v>
-      </c>
-      <c r="AP4">
-        <v>-4.2683999999999997</v>
-      </c>
-      <c r="AQ4">
-        <v>-4.3228999999999997</v>
-      </c>
-      <c r="AR4">
-        <v>-1.7878000000000001</v>
-      </c>
-      <c r="AS4">
-        <v>-1.5837000000000001</v>
-      </c>
-      <c r="AT4">
-        <v>-2.7273999999999998</v>
-      </c>
-      <c r="AU4">
-        <v>-2.3435000000000001</v>
-      </c>
-      <c r="AV4" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="AW4" s="7">
-        <v>598.66899999999998</v>
-      </c>
-      <c r="AX4" s="7">
-        <v>603.60720000000003</v>
-      </c>
-      <c r="AY4" s="7">
-        <v>609.09829999999999</v>
-      </c>
-      <c r="AZ4" s="7">
-        <v>609.57989999999995</v>
-      </c>
-      <c r="BA4" t="s">
-        <v>2</v>
-      </c>
-      <c r="BB4" s="13">
-        <v>-0.4531</v>
-      </c>
-      <c r="BC4" s="13">
-        <v>-1.329</v>
-      </c>
-      <c r="BD4">
-        <v>24.260100000000001</v>
-      </c>
-      <c r="BE4">
-        <v>22.967700000000001</v>
-      </c>
-      <c r="BF4" s="13">
-        <v>14.0365</v>
-      </c>
-      <c r="BG4" s="13">
-        <v>14.1881</v>
-      </c>
-      <c r="BH4">
-        <v>113.4755</v>
-      </c>
-      <c r="BI4">
-        <v>117.845</v>
-      </c>
-      <c r="BJ4" s="8">
-        <v>36.828099999999999</v>
-      </c>
-      <c r="BK4" s="8">
-        <v>37.734200000000001</v>
-      </c>
-      <c r="BL4" s="13">
-        <v>-1.0127999999999999</v>
-      </c>
-      <c r="BM4" s="13">
-        <v>-2.9868999999999999</v>
-      </c>
-      <c r="BN4">
-        <v>24.3781</v>
-      </c>
-      <c r="BO4">
-        <v>22.945399999999999</v>
-      </c>
-      <c r="BP4" s="13">
-        <v>14.832800000000001</v>
-      </c>
-      <c r="BQ4" s="13">
-        <v>13.7043</v>
-      </c>
-      <c r="BR4">
-        <v>105.47839999999999</v>
-      </c>
-      <c r="BS4">
-        <v>108.0421</v>
-      </c>
-      <c r="BT4" s="8">
-        <v>38.423299999999998</v>
-      </c>
-      <c r="BU4" s="8">
-        <v>37.145899999999997</v>
-      </c>
     </row>
-    <row r="5" spans="1:73">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1892,206 +1100,8 @@
       <c r="G5">
         <v>-34.453699999999998</v>
       </c>
-      <c r="H5">
-        <v>10.7966</v>
-      </c>
-      <c r="I5">
-        <v>10.3803</v>
-      </c>
-      <c r="J5">
-        <v>-32.269599999999997</v>
-      </c>
-      <c r="K5">
-        <v>-34.8917</v>
-      </c>
-      <c r="L5">
-        <v>9.4794</v>
-      </c>
-      <c r="M5">
-        <v>13.446300000000001</v>
-      </c>
-      <c r="N5">
-        <v>-9.7789999999999999</v>
-      </c>
-      <c r="O5">
-        <v>-11.3995</v>
-      </c>
-      <c r="P5">
-        <v>17.654199999999999</v>
-      </c>
-      <c r="Q5">
-        <v>18.137599999999999</v>
-      </c>
-      <c r="R5">
-        <v>-27.9268</v>
-      </c>
-      <c r="S5">
-        <v>-31.923100000000002</v>
-      </c>
-      <c r="T5">
-        <v>10.4917</v>
-      </c>
-      <c r="U5">
-        <v>12.026899999999999</v>
-      </c>
-      <c r="V5">
-        <v>-29.5398</v>
-      </c>
-      <c r="W5">
-        <v>-37.2849</v>
-      </c>
-      <c r="X5">
-        <v>9.2141000000000002</v>
-      </c>
-      <c r="Y5">
-        <v>13.035299999999999</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA5">
-        <v>-2.1999999999999999E-2</v>
-      </c>
-      <c r="AB5">
-        <v>-2.4199999999999999E-2</v>
-      </c>
-      <c r="AC5">
-        <v>0.34520000000000001</v>
-      </c>
-      <c r="AD5">
-        <v>0.34620000000000001</v>
-      </c>
-      <c r="AE5">
-        <v>-3.78E-2</v>
-      </c>
-      <c r="AF5">
-        <v>-3.3700000000000001E-2</v>
-      </c>
-      <c r="AG5">
-        <v>0.34460000000000002</v>
-      </c>
-      <c r="AH5">
-        <v>0.34189999999999998</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>55</v>
-      </c>
-      <c r="AJ5">
-        <v>-3.8399000000000001</v>
-      </c>
-      <c r="AK5">
-        <v>-3.9874000000000001</v>
-      </c>
-      <c r="AL5">
-        <v>-1.8320000000000001</v>
-      </c>
-      <c r="AM5">
-        <v>-2.0514000000000001</v>
-      </c>
-      <c r="AN5">
-        <v>-2.6448</v>
-      </c>
-      <c r="AO5">
-        <v>-2.5880000000000001</v>
-      </c>
-      <c r="AP5">
-        <v>-3.8351000000000002</v>
-      </c>
-      <c r="AQ5">
-        <v>-3.8904000000000001</v>
-      </c>
-      <c r="AR5">
-        <v>-1.8660000000000001</v>
-      </c>
-      <c r="AS5">
-        <v>-1.8758999999999999</v>
-      </c>
-      <c r="AT5">
-        <v>-2.3254000000000001</v>
-      </c>
-      <c r="AU5">
-        <v>-2.3121999999999998</v>
-      </c>
-      <c r="AV5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="AW5" s="7">
-        <v>702.67759999999998</v>
-      </c>
-      <c r="AX5" s="7">
-        <v>730.62710000000004</v>
-      </c>
-      <c r="AY5" s="7">
-        <v>686.63049999999998</v>
-      </c>
-      <c r="AZ5" s="7">
-        <v>686.62649999999996</v>
-      </c>
-      <c r="BA5" t="s">
-        <v>3</v>
-      </c>
-      <c r="BB5" s="13">
-        <v>7.8963999999999999</v>
-      </c>
-      <c r="BC5" s="13">
-        <v>6.4328000000000003</v>
-      </c>
-      <c r="BD5">
-        <v>25.956399999999999</v>
-      </c>
-      <c r="BE5">
-        <v>25.629899999999999</v>
-      </c>
-      <c r="BF5" s="13">
-        <v>14.8062</v>
-      </c>
-      <c r="BG5" s="13">
-        <v>11.571999999999999</v>
-      </c>
-      <c r="BH5">
-        <v>104.1074</v>
-      </c>
-      <c r="BI5">
-        <v>102.3282</v>
-      </c>
-      <c r="BJ5" s="8">
-        <v>41.295999999999999</v>
-      </c>
-      <c r="BK5" s="8">
-        <v>40.606400000000001</v>
-      </c>
-      <c r="BL5" s="13">
-        <v>7.4474</v>
-      </c>
-      <c r="BM5" s="13">
-        <v>4.0753000000000004</v>
-      </c>
-      <c r="BN5">
-        <v>25.253399999999999</v>
-      </c>
-      <c r="BO5">
-        <v>23.824100000000001</v>
-      </c>
-      <c r="BP5" s="13">
-        <v>15.7692</v>
-      </c>
-      <c r="BQ5" s="13">
-        <v>15.224600000000001</v>
-      </c>
-      <c r="BR5">
-        <v>100.7954</v>
-      </c>
-      <c r="BS5">
-        <v>101.61879999999999</v>
-      </c>
-      <c r="BT5" s="8">
-        <v>40.316200000000002</v>
-      </c>
-      <c r="BU5" s="8">
-        <v>39.437600000000003</v>
-      </c>
     </row>
-    <row r="6" spans="1:73">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -2113,206 +1123,8 @@
       <c r="G6">
         <v>-34.852600000000002</v>
       </c>
-      <c r="H6">
-        <v>10.8177</v>
-      </c>
-      <c r="I6">
-        <v>13.041499999999999</v>
-      </c>
-      <c r="J6">
-        <v>-32.376199999999997</v>
-      </c>
-      <c r="K6">
-        <v>-24.7942</v>
-      </c>
-      <c r="L6">
-        <v>5.6333000000000002</v>
-      </c>
-      <c r="M6">
-        <v>5.8731</v>
-      </c>
-      <c r="N6">
-        <v>-5.4283999999999999</v>
-      </c>
-      <c r="O6">
-        <v>-11.751200000000001</v>
-      </c>
-      <c r="P6">
-        <v>19.572500000000002</v>
-      </c>
-      <c r="Q6">
-        <v>20.8856</v>
-      </c>
-      <c r="R6">
-        <v>-30.3277</v>
-      </c>
-      <c r="S6">
-        <v>-23.183700000000002</v>
-      </c>
-      <c r="T6">
-        <v>10.530200000000001</v>
-      </c>
-      <c r="U6">
-        <v>13.0402</v>
-      </c>
-      <c r="V6">
-        <v>-21.195399999999999</v>
-      </c>
-      <c r="W6">
-        <v>-18.7562</v>
-      </c>
-      <c r="X6">
-        <v>4.3018000000000001</v>
-      </c>
-      <c r="Y6">
-        <v>5.2808000000000002</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>4</v>
-      </c>
-      <c r="AA6">
-        <v>-5.3499999999999999E-2</v>
-      </c>
-      <c r="AB6">
-        <v>-6.4199999999999993E-2</v>
-      </c>
-      <c r="AC6">
-        <v>0.4385</v>
-      </c>
-      <c r="AD6">
-        <v>0.4385</v>
-      </c>
-      <c r="AE6">
-        <v>-0.1104</v>
-      </c>
-      <c r="AF6">
-        <v>-0.10340000000000001</v>
-      </c>
-      <c r="AG6">
-        <v>0.39169999999999999</v>
-      </c>
-      <c r="AH6">
-        <v>0.37759999999999999</v>
-      </c>
-      <c r="AI6" t="s">
-        <v>56</v>
-      </c>
-      <c r="AJ6">
-        <v>-4.4505999999999997</v>
-      </c>
-      <c r="AK6">
-        <v>-4.2122000000000002</v>
-      </c>
-      <c r="AL6">
-        <v>-1.3866000000000001</v>
-      </c>
-      <c r="AM6">
-        <v>-1.4834000000000001</v>
-      </c>
-      <c r="AN6">
-        <v>-2.9053</v>
-      </c>
-      <c r="AO6">
-        <v>-2.6880999999999999</v>
-      </c>
-      <c r="AP6">
-        <v>-4.4263000000000003</v>
-      </c>
-      <c r="AQ6">
-        <v>-4.3144</v>
-      </c>
-      <c r="AR6">
-        <v>-1.1557999999999999</v>
-      </c>
-      <c r="AS6">
-        <v>-1.3996999999999999</v>
-      </c>
-      <c r="AT6">
-        <v>-2.5358000000000001</v>
-      </c>
-      <c r="AU6">
-        <v>-2.3426999999999998</v>
-      </c>
-      <c r="AV6" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="AW6" s="7">
-        <v>635.41880000000003</v>
-      </c>
-      <c r="AX6" s="7">
-        <v>643.58429999999998</v>
-      </c>
-      <c r="AY6" s="7">
-        <v>668.22439999999995</v>
-      </c>
-      <c r="AZ6" s="7">
-        <v>682.00959999999998</v>
-      </c>
-      <c r="BA6" t="s">
-        <v>4</v>
-      </c>
-      <c r="BB6" s="13">
-        <v>4.0837000000000003</v>
-      </c>
-      <c r="BC6" s="13">
-        <v>0.36399999999999999</v>
-      </c>
-      <c r="BD6">
-        <v>28.497299999999999</v>
-      </c>
-      <c r="BE6">
-        <v>25.174900000000001</v>
-      </c>
-      <c r="BF6" s="13">
-        <v>17.913699999999999</v>
-      </c>
-      <c r="BG6" s="13">
-        <v>16.572500000000002</v>
-      </c>
-      <c r="BH6">
-        <v>120.803</v>
-      </c>
-      <c r="BI6">
-        <v>116.639</v>
-      </c>
-      <c r="BJ6" s="8">
-        <v>38.438499999999998</v>
-      </c>
-      <c r="BK6" s="8">
-        <v>38.865900000000003</v>
-      </c>
-      <c r="BL6" s="13">
-        <v>1.8811</v>
-      </c>
-      <c r="BM6" s="13">
-        <v>1.5646</v>
-      </c>
-      <c r="BN6">
-        <v>23.291</v>
-      </c>
-      <c r="BO6">
-        <v>23.409400000000002</v>
-      </c>
-      <c r="BP6" s="13">
-        <v>15.4878</v>
-      </c>
-      <c r="BQ6" s="13">
-        <v>14.4129</v>
-      </c>
-      <c r="BR6">
-        <v>117.5744</v>
-      </c>
-      <c r="BS6">
-        <v>114.39490000000001</v>
-      </c>
-      <c r="BT6" s="8">
-        <v>34.999499999999998</v>
-      </c>
-      <c r="BU6" s="8">
-        <v>36.046599999999998</v>
-      </c>
     </row>
-    <row r="7" spans="1:73">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -2333,204 +1145,6 @@
       </c>
       <c r="G7">
         <v>-26.096499999999999</v>
-      </c>
-      <c r="H7">
-        <v>14.558</v>
-      </c>
-      <c r="I7">
-        <v>13.419700000000001</v>
-      </c>
-      <c r="J7">
-        <v>-40.521799999999999</v>
-      </c>
-      <c r="K7">
-        <v>-27.829000000000001</v>
-      </c>
-      <c r="L7">
-        <v>10.3948</v>
-      </c>
-      <c r="M7">
-        <v>10.1638</v>
-      </c>
-      <c r="N7">
-        <v>-9.1348000000000003</v>
-      </c>
-      <c r="O7">
-        <v>-13.7601</v>
-      </c>
-      <c r="P7">
-        <v>19.713699999999999</v>
-      </c>
-      <c r="Q7">
-        <v>20.383099999999999</v>
-      </c>
-      <c r="R7">
-        <v>-35.1312</v>
-      </c>
-      <c r="S7">
-        <v>-37.859000000000002</v>
-      </c>
-      <c r="T7">
-        <v>12.1767</v>
-      </c>
-      <c r="U7">
-        <v>12.527799999999999</v>
-      </c>
-      <c r="V7">
-        <v>-32.599200000000003</v>
-      </c>
-      <c r="W7">
-        <v>-23.528099999999998</v>
-      </c>
-      <c r="X7">
-        <v>12.318099999999999</v>
-      </c>
-      <c r="Y7">
-        <v>11.119300000000001</v>
-      </c>
-      <c r="Z7" t="s">
-        <v>5</v>
-      </c>
-      <c r="AA7">
-        <v>-0.1241</v>
-      </c>
-      <c r="AB7">
-        <v>-0.1164</v>
-      </c>
-      <c r="AC7">
-        <v>0.41710000000000003</v>
-      </c>
-      <c r="AD7">
-        <v>0.40610000000000002</v>
-      </c>
-      <c r="AE7">
-        <v>-9.4299999999999995E-2</v>
-      </c>
-      <c r="AF7">
-        <v>-9.7799999999999998E-2</v>
-      </c>
-      <c r="AG7">
-        <v>0.42720000000000002</v>
-      </c>
-      <c r="AH7">
-        <v>0.40820000000000001</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>57</v>
-      </c>
-      <c r="AJ7">
-        <v>-4.1776999999999997</v>
-      </c>
-      <c r="AK7">
-        <v>-4.3109999999999999</v>
-      </c>
-      <c r="AL7">
-        <v>-1.5572999999999999</v>
-      </c>
-      <c r="AM7">
-        <v>-1.8997999999999999</v>
-      </c>
-      <c r="AN7">
-        <v>-2.7261000000000002</v>
-      </c>
-      <c r="AO7">
-        <v>-2.4733999999999998</v>
-      </c>
-      <c r="AP7">
-        <v>-4.3122999999999996</v>
-      </c>
-      <c r="AQ7">
-        <v>-4.1980000000000004</v>
-      </c>
-      <c r="AR7">
-        <v>-1.891</v>
-      </c>
-      <c r="AS7">
-        <v>-2.0828000000000002</v>
-      </c>
-      <c r="AT7">
-        <v>-1.8732</v>
-      </c>
-      <c r="AU7">
-        <v>-1.5786</v>
-      </c>
-      <c r="AV7" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="AW7" s="7">
-        <v>731.71870000000001</v>
-      </c>
-      <c r="AX7" s="7">
-        <v>735.13980000000004</v>
-      </c>
-      <c r="AY7" s="7">
-        <v>680.21169999999995</v>
-      </c>
-      <c r="AZ7" s="7">
-        <v>678.05020000000002</v>
-      </c>
-      <c r="BA7" t="s">
-        <v>5</v>
-      </c>
-      <c r="BB7" s="13">
-        <v>-0.51700000000000002</v>
-      </c>
-      <c r="BC7" s="13">
-        <v>-0.30109999999999998</v>
-      </c>
-      <c r="BD7">
-        <v>23.6936</v>
-      </c>
-      <c r="BE7">
-        <v>24.040700000000001</v>
-      </c>
-      <c r="BF7" s="13">
-        <v>17.324400000000001</v>
-      </c>
-      <c r="BG7" s="13">
-        <v>15.9033</v>
-      </c>
-      <c r="BH7">
-        <v>117.788</v>
-      </c>
-      <c r="BI7">
-        <v>116.5749</v>
-      </c>
-      <c r="BJ7" s="8">
-        <v>40.414299999999997</v>
-      </c>
-      <c r="BK7" s="8">
-        <v>39.947299999999998</v>
-      </c>
-      <c r="BL7" s="13">
-        <v>-0.56530000000000002</v>
-      </c>
-      <c r="BM7" s="13">
-        <v>-1.379</v>
-      </c>
-      <c r="BN7">
-        <v>22.8567</v>
-      </c>
-      <c r="BO7">
-        <v>21.2927</v>
-      </c>
-      <c r="BP7" s="13">
-        <v>14.9474</v>
-      </c>
-      <c r="BQ7" s="13">
-        <v>12.110799999999999</v>
-      </c>
-      <c r="BR7">
-        <v>118.1288</v>
-      </c>
-      <c r="BS7">
-        <v>114.2012</v>
-      </c>
-      <c r="BT7" s="8">
-        <v>37.833799999999997</v>
-      </c>
-      <c r="BU7" s="8">
-        <v>34.575499999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>